<commit_message>
Add tests for staff changes and workplans functionality
- Implement StaffChangesTest to validate officer promotions, department changes, and access management.
- Create WorkplansTest to ensure Heads of Departments can prepare, submit, and revise workplans, including handling budget adjustments.
- Update HodTeamAndStaffTest to restrict staff list access for roles without permission, allowing only position changes for assistants.
- Modify PagesTest to clarify assistant access to the staff list, ensuring they can only record promotions and transfers.
</commit_message>
<xml_diff>
--- a/docs/guides/FAPM-Practice-Staff-List.xlsx
+++ b/docs/guides/FAPM-Practice-Staff-List.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>M&amp;E Officer</t>
+          <t>ICT Officer</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Monitoring &amp; Evaluation</t>
+          <t>ICT</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Monitoring &amp; Evaluation</t>
+          <t>ICT</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Monitoring &amp; Evaluation</t>
+          <t>ICT</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Monitoring &amp; Evaluation</t>
+          <t>ICT</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -874,6 +874,11 @@
           <t>Headquarters</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>mary.njeri@example.com</t>
+        </is>
+      </c>
       <c r="I9" s="2" t="n"/>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
@@ -884,10 +889,54 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>P90007</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Samuel Kiprono</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Permanent</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ICT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Headquarters</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>samuel.kiprono@example.com</t>
+        </is>
+      </c>
       <c r="I10" s="2" t="n"/>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n"/>

</xml_diff>